<commit_message>
Time video tracks with true frame times; script remaining quoted numbers
- video_analysis.py: damped-sine fits against true per-frame times (ffprobe);
  removes the 0.7-2.9% frequency outliers caused by variable frame rate
- check_video_clocks.py + Data/Video/frame_times/: per-file ffprobe check
- clock factor read from clock_calibration.json everywhere; mains line located in all 21 runs
- supporting_numbers.py: ADC step, noise, dipole moment/turns, air drag, time per read
- figures: proposed circuit relabelled with component values; nominal vs true rates
- CITATION.cff and .zenodo.json for archiving

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFRkKkuoXceM2uGC7BgjcC
</commit_message>
<xml_diff>
--- a/Data/Results/Overall_Results.xlsx
+++ b/Data/Results/Overall_Results.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per-run results" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Video tracks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -464,7 +465,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>10.84</v>
+        <v>10.83</v>
       </c>
       <c r="D2" t="n">
         <v>0.25</v>
@@ -473,7 +474,7 @@
         <v>603</v>
       </c>
       <c r="F2" t="n">
-        <v>2.0811</v>
+        <v>2.081</v>
       </c>
       <c r="G2" t="n">
         <v>17.71</v>
@@ -523,7 +524,7 @@
         <v>547</v>
       </c>
       <c r="F4" t="n">
-        <v>2.0811</v>
+        <v>2.081</v>
       </c>
       <c r="G4" t="n">
         <v>15.58</v>
@@ -548,7 +549,7 @@
         <v>541</v>
       </c>
       <c r="F5" t="n">
-        <v>2.0819</v>
+        <v>2.0818</v>
       </c>
       <c r="G5" t="n">
         <v>16.57</v>
@@ -598,7 +599,7 @@
         <v>556</v>
       </c>
       <c r="F7" t="n">
-        <v>2.0824</v>
+        <v>2.0823</v>
       </c>
       <c r="G7" t="n">
         <v>15.82</v>
@@ -648,7 +649,7 @@
         <v>525</v>
       </c>
       <c r="F9" t="n">
-        <v>2.0824</v>
+        <v>2.0823</v>
       </c>
       <c r="G9" t="n">
         <v>15.34</v>
@@ -673,7 +674,7 @@
         <v>567</v>
       </c>
       <c r="F10" t="n">
-        <v>2.0812</v>
+        <v>2.0811</v>
       </c>
       <c r="G10" t="n">
         <v>3.98</v>
@@ -714,7 +715,7 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>12.69</v>
+        <v>12.68</v>
       </c>
       <c r="D12" t="n">
         <v>0.12</v>
@@ -723,7 +724,7 @@
         <v>461</v>
       </c>
       <c r="F12" t="n">
-        <v>1.8624</v>
+        <v>1.8623</v>
       </c>
       <c r="G12" t="n">
         <v>13.71</v>
@@ -798,7 +799,7 @@
         <v>441</v>
       </c>
       <c r="F15" t="n">
-        <v>1.8624</v>
+        <v>1.8623</v>
       </c>
       <c r="G15" t="n">
         <v>14.13</v>
@@ -823,7 +824,7 @@
         <v>408</v>
       </c>
       <c r="F16" t="n">
-        <v>1.862</v>
+        <v>1.8619</v>
       </c>
       <c r="G16" t="n">
         <v>17.56</v>
@@ -848,7 +849,7 @@
         <v>443</v>
       </c>
       <c r="F17" t="n">
-        <v>1.8625</v>
+        <v>1.8624</v>
       </c>
       <c r="G17" t="n">
         <v>14.13</v>
@@ -898,7 +899,7 @@
         <v>601</v>
       </c>
       <c r="F19" t="n">
-        <v>2.0843</v>
+        <v>2.0842</v>
       </c>
       <c r="G19" t="n">
         <v>5.93</v>
@@ -948,7 +949,7 @@
         <v>427</v>
       </c>
       <c r="F21" t="n">
-        <v>1.8626</v>
+        <v>1.8625</v>
       </c>
       <c r="G21" t="n">
         <v>6.69</v>
@@ -973,7 +974,7 @@
         <v>422</v>
       </c>
       <c r="F22" t="n">
-        <v>1.8627</v>
+        <v>1.8626</v>
       </c>
       <c r="G22" t="n">
         <v>1.56</v>
@@ -990,7 +991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1017,7 +1018,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11.887</v>
+        <v>11.886</v>
       </c>
       <c r="C2" t="n">
         <v>13.491</v>
@@ -1043,10 +1044,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.0821</v>
+        <v>2.082</v>
       </c>
       <c r="C4" t="n">
-        <v>1.8622</v>
+        <v>1.8621</v>
       </c>
     </row>
     <row r="6">
@@ -1093,7 +1094,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Clock factor s (mains hum)</t>
+          <t>Clock factor s (mains hum): value, run sd, grid tolerance</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1101,6 +1102,860 @@
       </c>
       <c r="C9" t="n">
         <v>0.004654665303857302</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.01261340909091608</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Clock factor s (video, spring 1)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1.261816174701981</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0003175508263850613</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Clock factor s (video, spring 2)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1.261757450701093</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0001193110105422994</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Decay of the motion, spring 1 video (1e-3 /s): mean, sd</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11.30583301381962</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.3011073087573776</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>spring</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fps</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>frame_dt_sd_ms</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>f_even_spacing</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>gamma</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>gamma_se</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>late</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>A0_cm</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>resid_mm</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>passes_tracking_cut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WA0011</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>29.91380324359163</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1880837394898279</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2.080102097269879</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.080112606313174</v>
+      </c>
+      <c r="G2" t="n">
+        <v>11.38523115355167</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.2558378209883627</v>
+      </c>
+      <c r="I2" t="n">
+        <v>11.79284686202075</v>
+      </c>
+      <c r="J2" t="n">
+        <v>10.73563519563343</v>
+      </c>
+      <c r="K2" t="n">
+        <v>2.07916880182023</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1.027358307916629</v>
+      </c>
+      <c r="M2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>WA0012</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>27.89772989658942</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.5189152383895269</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.0810254584173</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.081558784475021</v>
+      </c>
+      <c r="G3" t="n">
+        <v>11.12891580620499</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.2545991394033396</v>
+      </c>
+      <c r="I3" t="n">
+        <v>11.72922028502643</v>
+      </c>
+      <c r="J3" t="n">
+        <v>10.77392842987272</v>
+      </c>
+      <c r="K3" t="n">
+        <v>2.195094997674113</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1.06017815796873</v>
+      </c>
+      <c r="M3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>WA0023</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>27.90666215999443</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.00669294552754987</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.861518333486415</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.861517898124768</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.934119496263231</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2.523733207327468</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-1.750974363710142</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5.87733522099379</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2.156170793540221</v>
+      </c>
+      <c r="L4" t="n">
+        <v>11.7612234636176</v>
+      </c>
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>WA0026</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>27.97884107248401</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.7333269014897937</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.86623263524893</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.861153793298071</v>
+      </c>
+      <c r="G5" t="n">
+        <v>8.004825022201794</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.9531004955706638</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.7577099002448535</v>
+      </c>
+      <c r="J5" t="n">
+        <v>11.70125624689886</v>
+      </c>
+      <c r="K5" t="n">
+        <v>2.58285287005392</v>
+      </c>
+      <c r="L5" t="n">
+        <v>4.737477518760378</v>
+      </c>
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WA0027</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>27.90665279461502</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.006773138767758142</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.861009952855612</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.861007238354647</v>
+      </c>
+      <c r="G6" t="n">
+        <v>8.338348613994167</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.319670018086459</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.6803678428902173</v>
+      </c>
+      <c r="J6" t="n">
+        <v>12.4674000451775</v>
+      </c>
+      <c r="K6" t="n">
+        <v>3.065213422574178</v>
+      </c>
+      <c r="L6" t="n">
+        <v>7.749717889596368</v>
+      </c>
+      <c r="M6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WA0029</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>28.15150765359514</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.9994281652079648</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.874828369572518</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.861293118629037</v>
+      </c>
+      <c r="G7" t="n">
+        <v>11.35347061575416</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.9673252509946887</v>
+      </c>
+      <c r="I7" t="n">
+        <v>12.94282439784622</v>
+      </c>
+      <c r="J7" t="n">
+        <v>12.08363800888128</v>
+      </c>
+      <c r="K7" t="n">
+        <v>3.138236563273058</v>
+      </c>
+      <c r="L7" t="n">
+        <v>5.547484360956074</v>
+      </c>
+      <c r="M7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WA0030</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>27.9066049822266</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.3507284632877259</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.082420566759927</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.082685906037198</v>
+      </c>
+      <c r="G8" t="n">
+        <v>11.16739467135823</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.157010170869286</v>
+      </c>
+      <c r="I8" t="n">
+        <v>11.43329839294446</v>
+      </c>
+      <c r="J8" t="n">
+        <v>10.66051601298301</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.1302981985485</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.6477984517538925</v>
+      </c>
+      <c r="M8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WA0031</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>27.90660099295292</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.3659081934019626</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.081226881195123</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2.081589306883665</v>
+      </c>
+      <c r="G9" t="n">
+        <v>11.74282750786622</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.1860193844677393</v>
+      </c>
+      <c r="I9" t="n">
+        <v>12.17275122226524</v>
+      </c>
+      <c r="J9" t="n">
+        <v>11.22434512303373</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.149551594097812</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.703092564560435</v>
+      </c>
+      <c r="M9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WA0033</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>28.73612622282041</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.226999936331596</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.14060911499073</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.081099342779063</v>
+      </c>
+      <c r="G10" t="n">
+        <v>11.67242738054804</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.2294054204125283</v>
+      </c>
+      <c r="I10" t="n">
+        <v>11.94480674547112</v>
+      </c>
+      <c r="J10" t="n">
+        <v>10.53892888586965</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.254298475522049</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.911045556563531</v>
+      </c>
+      <c r="M10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WA0034</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>27.8996193813277</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.3014165784442847</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2.079604402779143</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2.080025185895525</v>
+      </c>
+      <c r="G11" t="n">
+        <v>11.04159254611021</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.3501458955285221</v>
+      </c>
+      <c r="I11" t="n">
+        <v>10.46114140953589</v>
+      </c>
+      <c r="J11" t="n">
+        <v>10.30926961339291</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1.837642051085498</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1.212345137869034</v>
+      </c>
+      <c r="M11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WA0035</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="n">
+        <v>28.28106202417918</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.9612141713582758</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.88494573419115</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.861586357997898</v>
+      </c>
+      <c r="G12" t="n">
+        <v>11.45302893465136</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.3818115331224482</v>
+      </c>
+      <c r="I12" t="n">
+        <v>12.16625857601267</v>
+      </c>
+      <c r="J12" t="n">
+        <v>10.34922863840551</v>
+      </c>
+      <c r="K12" t="n">
+        <v>2.386437340056734</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1.636182262610446</v>
+      </c>
+      <c r="M12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WA0037</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>29.91428683659796</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.1939785019587298</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.861452719387539</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.86145263874729</v>
+      </c>
+      <c r="G13" t="n">
+        <v>8.198572589268435</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1.246671358718851</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1.816315587064502</v>
+      </c>
+      <c r="J13" t="n">
+        <v>11.64952554953291</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2.636195045000545</v>
+      </c>
+      <c r="L13" t="n">
+        <v>7.851189007453788</v>
+      </c>
+      <c r="M13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WA0038</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>28.93406427097163</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.207920945286401</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.83341816583336</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.861256362615152</v>
+      </c>
+      <c r="G14" t="n">
+        <v>10.85003877273764</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.4321820091367367</v>
+      </c>
+      <c r="I14" t="n">
+        <v>8.324705796313452</v>
+      </c>
+      <c r="J14" t="n">
+        <v>11.68990073287162</v>
+      </c>
+      <c r="K14" t="n">
+        <v>2.862287336800814</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2.369803410646882</v>
+      </c>
+      <c r="M14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WA0040</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>28.01253037608762</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.6350309594131571</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.868701448692987</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1.861635260170718</v>
+      </c>
+      <c r="G15" t="n">
+        <v>8.863952294487387</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1.015779398663373</v>
+      </c>
+      <c r="I15" t="n">
+        <v>7.933661030889617</v>
+      </c>
+      <c r="J15" t="n">
+        <v>10.87587098031433</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2.5564057764157</v>
+      </c>
+      <c r="L15" t="n">
+        <v>6.263075975815045</v>
+      </c>
+      <c r="M15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WA0041</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="n">
+        <v>28.62605904582695</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.169658605077802</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.864990745686898</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.861569172001935</v>
+      </c>
+      <c r="G16" t="n">
+        <v>11.33406033986752</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.9080729799587274</v>
+      </c>
+      <c r="I16" t="n">
+        <v>9.34147383531087</v>
+      </c>
+      <c r="J16" t="n">
+        <v>5.852623511249042</v>
+      </c>
+      <c r="K16" t="n">
+        <v>2.292891537665596</v>
+      </c>
+      <c r="L16" t="n">
+        <v>3.78862141800266</v>
+      </c>
+      <c r="M16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WA0042</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>28.13644057738513</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.7889548612099579</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2.097702719645361</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2.081215810495511</v>
+      </c>
+      <c r="G17" t="n">
+        <v>11.00244203109799</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.2750361013512996</v>
+      </c>
+      <c r="I17" t="n">
+        <v>11.44685832116974</v>
+      </c>
+      <c r="J17" t="n">
+        <v>10.70296879487962</v>
+      </c>
+      <c r="K17" t="n">
+        <v>2.198915700071954</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1.094496990995321</v>
+      </c>
+      <c r="M17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WA0043</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" t="n">
+        <v>27.97507992294129</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.4528454757386503</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1.866099058236422</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.861535130631029</v>
+      </c>
+      <c r="G18" t="n">
+        <v>11.38866287532606</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.1533427972004316</v>
+      </c>
+      <c r="I18" t="n">
+        <v>11.72284702959748</v>
+      </c>
+      <c r="J18" t="n">
+        <v>10.94980771169494</v>
+      </c>
+      <c r="K18" t="n">
+        <v>2.731968545595914</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.7658283673005529</v>
+      </c>
+      <c r="M18" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regenerate Overall_Results.xlsx with unrounded video clock factor
</commit_message>
<xml_diff>
--- a/Data/Results/Overall_Results.xlsx
+++ b/Data/Results/Overall_Results.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per-run results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Video tracks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Per-run results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Video tracks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1114,10 +1114,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.261816174701981</v>
+        <v>1.261807557954652</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0003175508263850613</v>
+        <v>0.0003175486578796247</v>
       </c>
     </row>
     <row r="11">
@@ -1127,10 +1127,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.261757450701093</v>
+        <v>1.261779638473547</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0001193110105422994</v>
+        <v>0.0001193131086044521</v>
       </c>
     </row>
     <row r="12">

</xml_diff>